<commit_message>
Updated To Do List
</commit_message>
<xml_diff>
--- a/To Do List.xlsx
+++ b/To Do List.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10613"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2FE9E02-77D4-5A4D-95C4-6FF548697C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BC4663D-1B1C-6B48-9005-E0FF1AC9C9E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2372,7 +2372,7 @@
       </c>
       <c r="C5" s="57">
         <f>SUM(tblToDoListMaster[Progress]) / COUNT(tblToDoListMaster[Progress])</f>
-        <v>0.21944444444444444</v>
+        <v>0.26666666666666666</v>
       </c>
       <c r="D5" s="57"/>
       <c r="E5" s="53">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="F5" s="54" t="str">
         <f ca="1">E5-TODAY() &amp; " days left"</f>
-        <v>22 days left</v>
+        <v>21 days left</v>
       </c>
       <c r="G5" s="51" t="s">
         <v>38</v>
@@ -2453,7 +2453,7 @@
       <c r="E9" s="38"/>
       <c r="F9" s="38">
         <f>SUM(tblToDoList1[Progress]) / COUNT(tblToDoList1[Progress])</f>
-        <v>0.31666666666666665</v>
+        <v>0.6</v>
       </c>
       <c r="G9" s="17"/>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="F5" s="45" t="str">
         <f ca="1">E5-TODAY() &amp; " days left"</f>
-        <v>12 days left</v>
+        <v>11 days left</v>
       </c>
       <c r="G5" s="30" t="s">
         <v>68</v>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="E8" s="38"/>
       <c r="F8" s="38">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
       <c r="G8" s="46" t="s">
         <v>73</v>
@@ -2802,7 +2802,7 @@
       </c>
       <c r="E9" s="38"/>
       <c r="F9" s="38">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="G9" s="17"/>
     </row>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="E11" s="38"/>
       <c r="F11" s="38">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G11" s="17"/>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="E12" s="38"/>
       <c r="F12" s="38">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G12" s="46"/>
     </row>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="E13" s="38"/>
       <c r="F13" s="38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="17"/>
     </row>
@@ -3072,7 +3072,7 @@
       </c>
       <c r="F5" s="45" t="str">
         <f ca="1">E5-TODAY() &amp; " days left"</f>
-        <v>18 days left</v>
+        <v>17 days left</v>
       </c>
       <c r="G5" s="30" t="s">
         <v>38</v>
@@ -3413,7 +3413,7 @@
       </c>
       <c r="F5" s="45" t="str">
         <f ca="1">E5-TODAY() &amp; " days left"</f>
-        <v>22 days left</v>
+        <v>21 days left</v>
       </c>
       <c r="G5" s="30" t="s">
         <v>38</v>
@@ -3737,7 +3737,7 @@
       </c>
       <c r="F5" s="45" t="str">
         <f ca="1">E5-TODAY() &amp; " days left"</f>
-        <v>25 days left</v>
+        <v>24 days left</v>
       </c>
       <c r="G5" s="30" t="s">
         <v>38</v>
@@ -4077,7 +4077,7 @@
       </c>
       <c r="F5" s="45" t="str">
         <f ca="1">E5-TODAY() &amp; " days left"</f>
-        <v>36 days left</v>
+        <v>35 days left</v>
       </c>
       <c r="G5" s="30" t="s">
         <v>38</v>

</xml_diff>